<commit_message>
Add PT2 blackbox repair support
</commit_message>
<xml_diff>
--- a/docs/hardware_l1_io_point_table_v1.xlsx
+++ b/docs/hardware_l1_io_point_table_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/promise/Downloads/3/Intership/ThreePhase_entier/Threephase_hardware/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F964B57-95B5-D44F-A53B-1C566CE23B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24961785-6C98-F846-AC79-A461D00CCE51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16040" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_总览" sheetId="1" r:id="rId1"/>
@@ -1293,9 +1293,6 @@
     <t>不能只把按钮等同 breaker_closed=true</t>
   </si>
   <si>
-    <t>L1-DI-G1-011</t>
-  </si>
-  <si>
     <t>Gen1 分闸按钮</t>
   </si>
   <si>
@@ -2146,9 +2143,6 @@
   </si>
   <si>
     <t>不能显示正常合闸；要求人工检查</t>
-  </si>
-  <si>
-    <t>合位和分位同时有效，状态灯进入告警态</t>
   </si>
   <si>
     <t>SAFE-007</t>
@@ -2495,6 +2489,14 @@
   </si>
   <si>
     <t>stop/manual/auto/invalid</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>L1-DI-G1-011</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>合位和分位同时有效，状态灯进入告警态</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -2502,7 +2504,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -2561,6 +2563,13 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F2933"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -2613,7 +2622,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2652,6 +2661,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3229,7 +3241,7 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" ht="20" customHeight="1">
       <c r="A23" s="4" t="s">
         <v>34</v>
       </c>
@@ -3246,7 +3258,7 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" ht="20" customHeight="1">
       <c r="A24" s="4" t="s">
         <v>36</v>
       </c>
@@ -3263,7 +3275,7 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" ht="20" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>38</v>
       </c>
@@ -3459,7 +3471,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" ht="25" customHeight="1">
       <c r="A14" s="5">
         <v>1</v>
       </c>
@@ -3473,7 +3485,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" ht="25" customHeight="1">
       <c r="A15" s="5">
         <v>2</v>
       </c>
@@ -3487,7 +3499,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="28">
+    <row r="16" spans="1:4" ht="25" customHeight="1">
       <c r="A16" s="5">
         <v>3</v>
       </c>
@@ -3501,7 +3513,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" ht="25" customHeight="1">
       <c r="A17" s="5">
         <v>4</v>
       </c>
@@ -3515,7 +3527,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" ht="25" customHeight="1">
       <c r="A18" s="5">
         <v>5</v>
       </c>
@@ -3529,7 +3541,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" ht="25" customHeight="1">
       <c r="A19" s="5">
         <v>6</v>
       </c>
@@ -5362,7 +5374,7 @@
         <v>27</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>416</v>
+        <v>815</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>104</v>
@@ -5374,7 +5386,7 @@
         <v>288</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>108</v>
@@ -5386,31 +5398,31 @@
         <v>215</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K31" s="4" t="s">
         <v>217</v>
       </c>
       <c r="L31" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="M31" s="4" t="s">
         <v>419</v>
       </c>
-      <c r="M31" s="4" t="s">
+      <c r="N31" s="4" t="s">
         <v>420</v>
       </c>
-      <c r="N31" s="4" t="s">
+      <c r="O31" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="O31" s="4" t="s">
+      <c r="P31" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="P31" s="4" t="s">
+      <c r="Q31" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="Q31" s="4" t="s">
+      <c r="R31" s="4" t="s">
         <v>424</v>
-      </c>
-      <c r="R31" s="4" t="s">
-        <v>425</v>
       </c>
       <c r="S31" s="7" t="s">
         <v>34</v>
@@ -5424,7 +5436,7 @@
         <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>104</v>
@@ -5436,43 +5448,43 @@
         <v>288</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>108</v>
       </c>
       <c r="H32" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="I32" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="J32" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="J32" s="4" t="s">
+      <c r="K32" s="4" t="s">
         <v>430</v>
       </c>
-      <c r="K32" s="4" t="s">
+      <c r="L32" s="4" t="s">
         <v>431</v>
       </c>
-      <c r="L32" s="4" t="s">
+      <c r="M32" s="4" t="s">
         <v>432</v>
       </c>
-      <c r="M32" s="4" t="s">
+      <c r="N32" s="4" t="s">
         <v>433</v>
       </c>
-      <c r="N32" s="4" t="s">
+      <c r="O32" s="4" t="s">
         <v>434</v>
       </c>
-      <c r="O32" s="4" t="s">
+      <c r="P32" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="P32" s="4" t="s">
+      <c r="Q32" s="4" t="s">
         <v>436</v>
       </c>
-      <c r="Q32" s="4" t="s">
+      <c r="R32" s="4" t="s">
         <v>437</v>
-      </c>
-      <c r="R32" s="4" t="s">
-        <v>438</v>
       </c>
       <c r="S32" s="7" t="s">
         <v>34</v>
@@ -5486,7 +5498,7 @@
         <v>29</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>199</v>
@@ -5498,43 +5510,43 @@
         <v>288</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>108</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I33" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="J33" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="J33" s="4" t="s">
+      <c r="K33" s="4" t="s">
         <v>442</v>
       </c>
-      <c r="K33" s="4" t="s">
+      <c r="L33" s="4" t="s">
         <v>443</v>
       </c>
-      <c r="L33" s="4" t="s">
+      <c r="M33" s="4" t="s">
         <v>444</v>
       </c>
-      <c r="M33" s="4" t="s">
+      <c r="N33" s="4" t="s">
         <v>445</v>
       </c>
-      <c r="N33" s="4" t="s">
+      <c r="O33" s="4" t="s">
         <v>446</v>
       </c>
-      <c r="O33" s="4" t="s">
+      <c r="P33" s="4" t="s">
         <v>447</v>
       </c>
-      <c r="P33" s="4" t="s">
+      <c r="Q33" s="4" t="s">
         <v>448</v>
       </c>
-      <c r="Q33" s="4" t="s">
+      <c r="R33" s="4" t="s">
         <v>449</v>
-      </c>
-      <c r="R33" s="4" t="s">
-        <v>450</v>
       </c>
       <c r="S33" s="7" t="s">
         <v>36</v>
@@ -5548,7 +5560,7 @@
         <v>30</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>104</v>
@@ -5560,43 +5572,43 @@
         <v>288</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>138</v>
       </c>
       <c r="H34" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="I34" s="4" t="s">
         <v>453</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="J34" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="J34" s="4" t="s">
+      <c r="K34" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="K34" s="4" t="s">
+      <c r="L34" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="L34" s="4" t="s">
+      <c r="M34" s="4" t="s">
         <v>457</v>
       </c>
-      <c r="M34" s="4" t="s">
+      <c r="N34" s="4" t="s">
         <v>458</v>
       </c>
-      <c r="N34" s="4" t="s">
+      <c r="O34" s="4" t="s">
         <v>459</v>
       </c>
-      <c r="O34" s="4" t="s">
+      <c r="P34" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="P34" s="4" t="s">
+      <c r="Q34" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="Q34" s="4" t="s">
+      <c r="R34" s="4" t="s">
         <v>462</v>
-      </c>
-      <c r="R34" s="4" t="s">
-        <v>463</v>
       </c>
       <c r="S34" s="7" t="s">
         <v>34</v>
@@ -5610,7 +5622,7 @@
         <v>31</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>104</v>
@@ -5622,43 +5634,43 @@
         <v>288</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>138</v>
       </c>
       <c r="H35" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="I35" s="4" t="s">
         <v>466</v>
       </c>
-      <c r="I35" s="4" t="s">
+      <c r="J35" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="J35" s="4" t="s">
+      <c r="K35" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="L35" s="4" t="s">
         <v>468</v>
       </c>
-      <c r="K35" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="L35" s="4" t="s">
+      <c r="M35" s="4" t="s">
         <v>469</v>
       </c>
-      <c r="M35" s="4" t="s">
+      <c r="N35" s="4" t="s">
         <v>470</v>
       </c>
-      <c r="N35" s="4" t="s">
+      <c r="O35" s="4" t="s">
         <v>471</v>
       </c>
-      <c r="O35" s="4" t="s">
+      <c r="P35" s="4" t="s">
         <v>472</v>
       </c>
-      <c r="P35" s="4" t="s">
+      <c r="Q35" s="4" t="s">
         <v>473</v>
       </c>
-      <c r="Q35" s="4" t="s">
+      <c r="R35" s="4" t="s">
         <v>474</v>
-      </c>
-      <c r="R35" s="4" t="s">
-        <v>475</v>
       </c>
       <c r="S35" s="7" t="s">
         <v>38</v>
@@ -5672,7 +5684,7 @@
         <v>32</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>104</v>
@@ -5684,7 +5696,7 @@
         <v>288</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>138</v>
@@ -5693,34 +5705,34 @@
         <v>139</v>
       </c>
       <c r="I36" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="J36" s="4" t="s">
         <v>478</v>
-      </c>
-      <c r="J36" s="4" t="s">
-        <v>479</v>
       </c>
       <c r="K36" s="4" t="s">
         <v>154</v>
       </c>
       <c r="L36" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="M36" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="N36" s="4" t="s">
         <v>480</v>
       </c>
-      <c r="M36" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="N36" s="4" t="s">
+      <c r="O36" s="4" t="s">
         <v>481</v>
       </c>
-      <c r="O36" s="4" t="s">
+      <c r="P36" s="4" t="s">
         <v>482</v>
       </c>
-      <c r="P36" s="4" t="s">
+      <c r="Q36" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="Q36" s="4" t="s">
+      <c r="R36" s="4" t="s">
         <v>484</v>
-      </c>
-      <c r="R36" s="4" t="s">
-        <v>485</v>
       </c>
       <c r="S36" s="7" t="s">
         <v>34</v>
@@ -5734,7 +5746,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>104</v>
@@ -5746,43 +5758,43 @@
         <v>288</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>138</v>
       </c>
       <c r="H37" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="I37" s="4" t="s">
         <v>488</v>
       </c>
-      <c r="I37" s="4" t="s">
+      <c r="J37" s="4" t="s">
         <v>489</v>
-      </c>
-      <c r="J37" s="4" t="s">
-        <v>490</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>154</v>
       </c>
       <c r="L37" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="M37" s="4" t="s">
         <v>491</v>
       </c>
-      <c r="M37" s="4" t="s">
+      <c r="N37" s="4" t="s">
         <v>492</v>
       </c>
-      <c r="N37" s="4" t="s">
+      <c r="O37" s="4" t="s">
         <v>493</v>
       </c>
-      <c r="O37" s="4" t="s">
+      <c r="P37" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="P37" s="4" t="s">
+      <c r="Q37" s="4" t="s">
         <v>495</v>
       </c>
-      <c r="Q37" s="4" t="s">
+      <c r="R37" s="4" t="s">
         <v>496</v>
-      </c>
-      <c r="R37" s="4" t="s">
-        <v>497</v>
       </c>
       <c r="S37" s="7" t="s">
         <v>36</v>
@@ -5796,7 +5808,7 @@
         <v>34</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>104</v>
@@ -5805,10 +5817,10 @@
         <v>105</v>
       </c>
       <c r="E38" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="F38" s="4" t="s">
         <v>499</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>500</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>108</v>
@@ -5829,10 +5841,10 @@
         <v>293</v>
       </c>
       <c r="M38" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="N38" s="4" t="s">
         <v>501</v>
-      </c>
-      <c r="N38" s="4" t="s">
-        <v>502</v>
       </c>
       <c r="O38" s="4" t="s">
         <v>296</v>
@@ -5858,7 +5870,7 @@
         <v>35</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>104</v>
@@ -5867,10 +5879,10 @@
         <v>105</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>108</v>
@@ -5891,10 +5903,10 @@
         <v>305</v>
       </c>
       <c r="M39" s="4" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="N39" s="4" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="O39" s="4" t="s">
         <v>307</v>
@@ -5920,7 +5932,7 @@
         <v>36</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>312</v>
@@ -5929,10 +5941,10 @@
         <v>313</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>108</v>
@@ -5953,10 +5965,10 @@
         <v>318</v>
       </c>
       <c r="M40" s="4" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="N40" s="4" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="O40" s="4" t="s">
         <v>320</v>
@@ -5982,7 +5994,7 @@
         <v>37</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>104</v>
@@ -5991,10 +6003,10 @@
         <v>105</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>108</v>
@@ -6015,10 +6027,10 @@
         <v>328</v>
       </c>
       <c r="M41" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="N41" s="4" t="s">
         <v>511</v>
-      </c>
-      <c r="N41" s="4" t="s">
-        <v>512</v>
       </c>
       <c r="O41" s="4" t="s">
         <v>331</v>
@@ -6044,7 +6056,7 @@
         <v>38</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>104</v>
@@ -6053,10 +6065,10 @@
         <v>105</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>108</v>
@@ -6077,10 +6089,10 @@
         <v>340</v>
       </c>
       <c r="M42" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="N42" s="4" t="s">
         <v>515</v>
-      </c>
-      <c r="N42" s="4" t="s">
-        <v>516</v>
       </c>
       <c r="O42" s="4" t="s">
         <v>343</v>
@@ -6106,7 +6118,7 @@
         <v>39</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>104</v>
@@ -6115,10 +6127,10 @@
         <v>105</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>108</v>
@@ -6139,10 +6151,10 @@
         <v>353</v>
       </c>
       <c r="M43" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="N43" s="4" t="s">
         <v>519</v>
-      </c>
-      <c r="N43" s="4" t="s">
-        <v>520</v>
       </c>
       <c r="O43" s="4" t="s">
         <v>356</v>
@@ -6168,7 +6180,7 @@
         <v>40</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>104</v>
@@ -6177,10 +6189,10 @@
         <v>136</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>138</v>
@@ -6201,10 +6213,10 @@
         <v>364</v>
       </c>
       <c r="M44" s="4" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="N44" s="4" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="O44" s="4" t="s">
         <v>366</v>
@@ -6230,7 +6242,7 @@
         <v>41</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>104</v>
@@ -6239,10 +6251,10 @@
         <v>105</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>108</v>
@@ -6263,10 +6275,10 @@
         <v>376</v>
       </c>
       <c r="M45" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="N45" s="4" t="s">
         <v>526</v>
-      </c>
-      <c r="N45" s="4" t="s">
-        <v>527</v>
       </c>
       <c r="O45" s="4" t="s">
         <v>379</v>
@@ -6292,7 +6304,7 @@
         <v>42</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>199</v>
@@ -6301,10 +6313,10 @@
         <v>136</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>108</v>
@@ -6325,10 +6337,10 @@
         <v>388</v>
       </c>
       <c r="M46" s="4" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="N46" s="4" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="O46" s="4" t="s">
         <v>390</v>
@@ -6354,7 +6366,7 @@
         <v>43</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>104</v>
@@ -6363,10 +6375,10 @@
         <v>105</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>108</v>
@@ -6387,10 +6399,10 @@
         <v>399</v>
       </c>
       <c r="M47" s="4" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="N47" s="4" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="O47" s="4" t="s">
         <v>401</v>
@@ -6416,7 +6428,7 @@
         <v>44</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>104</v>
@@ -6425,10 +6437,10 @@
         <v>105</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>108</v>
@@ -6449,10 +6461,10 @@
         <v>409</v>
       </c>
       <c r="M48" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="N48" s="4" t="s">
         <v>536</v>
-      </c>
-      <c r="N48" s="4" t="s">
-        <v>537</v>
       </c>
       <c r="O48" s="4" t="s">
         <v>412</v>
@@ -6478,7 +6490,7 @@
         <v>45</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>104</v>
@@ -6487,10 +6499,10 @@
         <v>105</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>108</v>
@@ -6502,31 +6514,31 @@
         <v>215</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K49" s="4" t="s">
         <v>217</v>
       </c>
       <c r="L49" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="M49" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="N49" s="4" t="s">
         <v>540</v>
       </c>
-      <c r="N49" s="4" t="s">
-        <v>541</v>
-      </c>
       <c r="O49" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="P49" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="P49" s="4" t="s">
+      <c r="Q49" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="Q49" s="4" t="s">
+      <c r="R49" s="4" t="s">
         <v>424</v>
-      </c>
-      <c r="R49" s="4" t="s">
-        <v>425</v>
       </c>
       <c r="S49" s="7" t="s">
         <v>34</v>
@@ -6540,7 +6552,7 @@
         <v>46</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>104</v>
@@ -6549,46 +6561,46 @@
         <v>105</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="G50" s="5" t="s">
         <v>108</v>
       </c>
       <c r="H50" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="I50" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="I50" s="4" t="s">
+      <c r="J50" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="J50" s="4" t="s">
+      <c r="K50" s="4" t="s">
         <v>430</v>
       </c>
-      <c r="K50" s="4" t="s">
+      <c r="L50" s="4" t="s">
         <v>431</v>
       </c>
-      <c r="L50" s="4" t="s">
-        <v>432</v>
-      </c>
       <c r="M50" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="N50" s="4" t="s">
         <v>544</v>
       </c>
-      <c r="N50" s="4" t="s">
-        <v>545</v>
-      </c>
       <c r="O50" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="P50" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="P50" s="4" t="s">
+      <c r="Q50" s="4" t="s">
         <v>436</v>
       </c>
-      <c r="Q50" s="4" t="s">
+      <c r="R50" s="4" t="s">
         <v>437</v>
-      </c>
-      <c r="R50" s="4" t="s">
-        <v>438</v>
       </c>
       <c r="S50" s="7" t="s">
         <v>34</v>
@@ -6602,7 +6614,7 @@
         <v>47</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>199</v>
@@ -6611,46 +6623,46 @@
         <v>136</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>108</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I51" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="J51" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="J51" s="4" t="s">
+      <c r="K51" s="4" t="s">
         <v>442</v>
       </c>
-      <c r="K51" s="4" t="s">
+      <c r="L51" s="4" t="s">
         <v>443</v>
       </c>
-      <c r="L51" s="4" t="s">
-        <v>444</v>
-      </c>
       <c r="M51" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="N51" s="4" t="s">
         <v>548</v>
       </c>
-      <c r="N51" s="4" t="s">
-        <v>549</v>
-      </c>
       <c r="O51" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="P51" s="4" t="s">
         <v>447</v>
       </c>
-      <c r="P51" s="4" t="s">
+      <c r="Q51" s="4" t="s">
         <v>448</v>
       </c>
-      <c r="Q51" s="4" t="s">
+      <c r="R51" s="4" t="s">
         <v>449</v>
-      </c>
-      <c r="R51" s="4" t="s">
-        <v>450</v>
       </c>
       <c r="S51" s="7" t="s">
         <v>36</v>
@@ -6664,7 +6676,7 @@
         <v>48</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>104</v>
@@ -6673,46 +6685,46 @@
         <v>105</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="G52" s="5" t="s">
         <v>138</v>
       </c>
       <c r="H52" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="I52" s="4" t="s">
         <v>453</v>
       </c>
-      <c r="I52" s="4" t="s">
+      <c r="J52" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="J52" s="4" t="s">
+      <c r="K52" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="K52" s="4" t="s">
+      <c r="L52" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="L52" s="4" t="s">
+      <c r="M52" s="4" t="s">
         <v>457</v>
       </c>
-      <c r="M52" s="4" t="s">
-        <v>458</v>
-      </c>
       <c r="N52" s="4" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="O52" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="P52" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="P52" s="4" t="s">
+      <c r="Q52" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="Q52" s="4" t="s">
+      <c r="R52" s="4" t="s">
         <v>462</v>
-      </c>
-      <c r="R52" s="4" t="s">
-        <v>463</v>
       </c>
       <c r="S52" s="7" t="s">
         <v>34</v>
@@ -6726,7 +6738,7 @@
         <v>49</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>104</v>
@@ -6735,46 +6747,46 @@
         <v>105</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>138</v>
       </c>
       <c r="H53" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="I53" s="4" t="s">
         <v>466</v>
       </c>
-      <c r="I53" s="4" t="s">
+      <c r="J53" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="J53" s="4" t="s">
+      <c r="K53" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="L53" s="4" t="s">
         <v>468</v>
       </c>
-      <c r="K53" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="L53" s="4" t="s">
+      <c r="M53" s="4" t="s">
         <v>469</v>
       </c>
-      <c r="M53" s="4" t="s">
-        <v>470</v>
-      </c>
       <c r="N53" s="4" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="O53" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="P53" s="4" t="s">
         <v>472</v>
       </c>
-      <c r="P53" s="4" t="s">
+      <c r="Q53" s="4" t="s">
         <v>473</v>
       </c>
-      <c r="Q53" s="4" t="s">
+      <c r="R53" s="4" t="s">
         <v>474</v>
-      </c>
-      <c r="R53" s="4" t="s">
-        <v>475</v>
       </c>
       <c r="S53" s="7" t="s">
         <v>38</v>
@@ -6788,7 +6800,7 @@
         <v>50</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>104</v>
@@ -6797,10 +6809,10 @@
         <v>136</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="G54" s="5" t="s">
         <v>138</v>
@@ -6809,34 +6821,34 @@
         <v>139</v>
       </c>
       <c r="I54" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="J54" s="4" t="s">
         <v>478</v>
-      </c>
-      <c r="J54" s="4" t="s">
-        <v>479</v>
       </c>
       <c r="K54" s="4" t="s">
         <v>154</v>
       </c>
       <c r="L54" s="4" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="M54" s="4" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="N54" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="O54" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="P54" s="4" t="s">
         <v>482</v>
       </c>
-      <c r="P54" s="4" t="s">
+      <c r="Q54" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="Q54" s="4" t="s">
+      <c r="R54" s="4" t="s">
         <v>484</v>
-      </c>
-      <c r="R54" s="4" t="s">
-        <v>485</v>
       </c>
       <c r="S54" s="7" t="s">
         <v>34</v>
@@ -6850,7 +6862,7 @@
         <v>51</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C55" s="5" t="s">
         <v>104</v>
@@ -6859,46 +6871,46 @@
         <v>136</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="G55" s="5" t="s">
         <v>138</v>
       </c>
       <c r="H55" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="I55" s="4" t="s">
         <v>488</v>
       </c>
-      <c r="I55" s="4" t="s">
+      <c r="J55" s="4" t="s">
         <v>489</v>
-      </c>
-      <c r="J55" s="4" t="s">
-        <v>490</v>
       </c>
       <c r="K55" s="4" t="s">
         <v>154</v>
       </c>
       <c r="L55" s="4" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="M55" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="N55" s="4" t="s">
         <v>561</v>
       </c>
-      <c r="N55" s="4" t="s">
-        <v>562</v>
-      </c>
       <c r="O55" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="P55" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="P55" s="4" t="s">
+      <c r="Q55" s="4" t="s">
         <v>495</v>
       </c>
-      <c r="Q55" s="4" t="s">
+      <c r="R55" s="4" t="s">
         <v>496</v>
-      </c>
-      <c r="R55" s="4" t="s">
-        <v>497</v>
       </c>
       <c r="S55" s="7" t="s">
         <v>36</v>
@@ -6912,7 +6924,7 @@
         <v>52</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>312</v>
@@ -6921,46 +6933,46 @@
         <v>313</v>
       </c>
       <c r="E56" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="F56" s="4" t="s">
         <v>564</v>
-      </c>
-      <c r="F56" s="4" t="s">
-        <v>565</v>
       </c>
       <c r="G56" s="5" t="s">
         <v>108</v>
       </c>
       <c r="H56" s="5" t="s">
+        <v>565</v>
+      </c>
+      <c r="I56" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="I56" s="4" t="s">
+      <c r="J56" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="J56" s="4" t="s">
+      <c r="K56" s="4" t="s">
         <v>568</v>
       </c>
-      <c r="K56" s="4" t="s">
+      <c r="L56" s="4" t="s">
         <v>569</v>
       </c>
-      <c r="L56" s="4" t="s">
+      <c r="M56" s="4" t="s">
         <v>570</v>
       </c>
-      <c r="M56" s="4" t="s">
+      <c r="N56" s="4" t="s">
         <v>571</v>
       </c>
-      <c r="N56" s="4" t="s">
+      <c r="O56" s="4" t="s">
         <v>572</v>
       </c>
-      <c r="O56" s="4" t="s">
+      <c r="P56" s="4" t="s">
         <v>573</v>
       </c>
-      <c r="P56" s="4" t="s">
+      <c r="Q56" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="Q56" s="4" t="s">
+      <c r="R56" s="4" t="s">
         <v>575</v>
-      </c>
-      <c r="R56" s="4" t="s">
-        <v>576</v>
       </c>
       <c r="S56" s="7" t="s">
         <v>38</v>
@@ -6974,7 +6986,7 @@
         <v>53</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C57" s="5" t="s">
         <v>312</v>
@@ -6983,10 +6995,10 @@
         <v>313</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="G57" s="5" t="s">
         <v>138</v>
@@ -7004,25 +7016,25 @@
         <v>154</v>
       </c>
       <c r="L57" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="M57" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="M57" s="4" t="s">
+      <c r="N57" s="4" t="s">
         <v>580</v>
       </c>
-      <c r="N57" s="4" t="s">
+      <c r="O57" s="4" t="s">
         <v>581</v>
       </c>
-      <c r="O57" s="4" t="s">
+      <c r="P57" s="4" t="s">
         <v>582</v>
       </c>
-      <c r="P57" s="4" t="s">
+      <c r="Q57" s="4" t="s">
         <v>583</v>
       </c>
-      <c r="Q57" s="4" t="s">
+      <c r="R57" s="4" t="s">
         <v>584</v>
-      </c>
-      <c r="R57" s="4" t="s">
-        <v>585</v>
       </c>
       <c r="S57" s="7" t="s">
         <v>38</v>
@@ -7036,7 +7048,7 @@
         <v>54</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>199</v>
@@ -7045,46 +7057,46 @@
         <v>136</v>
       </c>
       <c r="E58" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F58" s="4" t="s">
         <v>587</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>588</v>
       </c>
       <c r="G58" s="5" t="s">
         <v>108</v>
       </c>
       <c r="H58" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="I58" s="4" t="s">
         <v>589</v>
       </c>
-      <c r="I58" s="4" t="s">
+      <c r="J58" s="4" t="s">
         <v>590</v>
       </c>
-      <c r="J58" s="4" t="s">
+      <c r="K58" s="4" t="s">
         <v>591</v>
       </c>
-      <c r="K58" s="4" t="s">
+      <c r="L58" s="4" t="s">
         <v>592</v>
       </c>
-      <c r="L58" s="4" t="s">
+      <c r="M58" s="4" t="s">
         <v>593</v>
       </c>
-      <c r="M58" s="4" t="s">
+      <c r="N58" s="4" t="s">
         <v>594</v>
       </c>
-      <c r="N58" s="4" t="s">
+      <c r="O58" s="4" t="s">
         <v>595</v>
       </c>
-      <c r="O58" s="4" t="s">
+      <c r="P58" s="4" t="s">
         <v>596</v>
       </c>
-      <c r="P58" s="4" t="s">
+      <c r="Q58" s="4" t="s">
         <v>597</v>
       </c>
-      <c r="Q58" s="4" t="s">
+      <c r="R58" s="4" t="s">
         <v>598</v>
-      </c>
-      <c r="R58" s="4" t="s">
-        <v>599</v>
       </c>
       <c r="S58" s="7" t="s">
         <v>38</v>
@@ -7118,27 +7130,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="34.5" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -7156,382 +7168,382 @@
     </row>
     <row r="4" spans="1:6" ht="31.5" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>602</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>603</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>604</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>605</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>606</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>607</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>608</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>610</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>611</v>
       </c>
-      <c r="F5" s="4" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>612</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>613</v>
-      </c>
       <c r="C6" s="4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>126</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F6" s="4" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>614</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>615</v>
       </c>
-      <c r="C7" s="4" t="s">
+    </row>
+    <row r="8" spans="1:6" ht="30" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>610</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>611</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>617</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>611</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28">
+    <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>618</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>619</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>263</v>
       </c>
       <c r="F9" s="4" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>620</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>814</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>621</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="F10" s="4" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>816</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>622</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>623</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>624</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="F11" s="4" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="30" customHeight="1">
+      <c r="A12" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>626</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="30" customHeight="1">
+      <c r="A13" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>625</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>626</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="28">
-      <c r="A12" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>627</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="E13" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="30" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>628</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>629</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="28">
-      <c r="A13" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>631</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>632</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>633</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="28">
-      <c r="A14" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>634</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>635</v>
       </c>
-      <c r="F14" s="4" t="s">
+    </row>
+    <row r="15" spans="1:6" ht="30" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>636</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="28">
-      <c r="A15" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>813</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>637</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>815</v>
-      </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>638</v>
       </c>
-      <c r="F15" s="4" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="30" customHeight="1">
+      <c r="A16" s="4" t="s">
         <v>639</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="28">
-      <c r="A16" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>640</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>641</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>642</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>643</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>644</v>
       </c>
-      <c r="F16" s="4" t="s">
+    </row>
+    <row r="17" spans="1:6" ht="30" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>639</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="28">
-      <c r="A17" s="4" t="s">
-        <v>640</v>
-      </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>642</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>646</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="F17" s="4" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="30" customHeight="1">
+      <c r="A18" s="4" t="s">
+        <v>639</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>648</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>642</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>643</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>647</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="28">
-      <c r="A18" s="4" t="s">
-        <v>640</v>
-      </c>
-      <c r="B18" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>649</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="F18" s="4" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="30" customHeight="1">
+      <c r="A19" s="4" t="s">
+        <v>639</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>642</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>643</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>650</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="28">
-      <c r="A19" s="4" t="s">
-        <v>640</v>
-      </c>
-      <c r="B19" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>652</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>642</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>643</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>653</v>
       </c>
-      <c r="F19" s="4" t="s">
+    </row>
+    <row r="20" spans="1:6" ht="30" customHeight="1">
+      <c r="A20" s="4" t="s">
         <v>654</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="4" t="s">
+      <c r="B20" s="4" t="s">
         <v>655</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>656</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="E20" s="4" t="s">
         <v>657</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="E20" s="4" t="s">
+      <c r="F20" s="4" t="s">
         <v>658</v>
       </c>
-      <c r="F20" s="4" t="s">
+    </row>
+    <row r="21" spans="1:6" ht="30" customHeight="1">
+      <c r="A21" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>659</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="4" t="s">
-        <v>655</v>
-      </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="4" t="s">
+        <v>656</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>660</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>657</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="E21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>661</v>
       </c>
-      <c r="F21" s="4" t="s">
+    </row>
+    <row r="22" spans="1:6" ht="30" customHeight="1">
+      <c r="A22" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>662</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="4" t="s">
-        <v>655</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>663</v>
-      </c>
       <c r="C22" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>154</v>
       </c>
       <c r="E22" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>664</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>665</v>
       </c>
     </row>
   </sheetData>
@@ -7558,24 +7570,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="34.5" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -7591,16 +7603,16 @@
     </row>
     <row r="4" spans="1:5" ht="31.5" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>668</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>669</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>670</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>671</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>63</v>
@@ -7608,172 +7620,172 @@
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>672</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>673</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>674</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>675</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>676</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>677</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>678</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>679</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>680</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>681</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>682</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>683</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>684</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>685</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>686</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>687</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>688</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>689</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>690</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>691</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>691</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>692</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>693</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>694</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>695</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>697</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>698</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>699</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>700</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>701</v>
+      <c r="E10" s="15" t="s">
+        <v>816</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>701</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>702</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>703</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>704</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>705</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="30" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>705</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>707</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>708</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>709</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>710</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>711</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="30" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>710</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>711</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>712</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>713</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>714</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>715</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>716</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" customHeight="1">
       <c r="A14" s="4" t="s">
+        <v>715</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>716</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>717</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>718</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>719</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>720</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>721</v>
       </c>
     </row>
   </sheetData>
@@ -7801,27 +7813,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="34.5" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -7839,262 +7851,262 @@
     </row>
     <row r="4" spans="1:6" ht="31.5" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>722</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>724</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>725</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>726</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>727</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>728</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>728</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>729</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>730</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>731</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>732</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>733</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>734</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>735</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>735</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>736</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>737</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>738</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>739</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>740</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>741</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>741</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>742</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>743</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>744</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>745</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>746</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>746</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>747</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>748</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>749</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>750</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>751</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>752</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>751</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>752</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>753</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>748</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>754</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>755</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>750</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>756</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>757</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>756</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>757</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>741</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>758</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>759</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>743</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>760</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>761</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>762</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>761</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>762</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>763</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>764</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>765</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="F11" s="4" t="s">
         <v>766</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>767</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>768</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>767</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>768</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>769</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="D12" s="4" t="s">
+        <v>764</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>770</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>771</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>766</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>772</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>772</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>773</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>774</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>775</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>776</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>777</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>778</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>779</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="4" t="s">
+        <v>778</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>779</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>780</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>781</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>782</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>783</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>784</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>785</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1">
       <c r="A15" s="4" t="s">
+        <v>784</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>785</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>786</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>787</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>788</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>789</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>790</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="4" t="s">
+        <v>790</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>716</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>791</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>792</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>718</v>
-      </c>
-      <c r="C16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>793</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>794</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>795</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>796</v>
       </c>
     </row>
   </sheetData>
@@ -8118,15 +8130,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="34.5" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B2" s="10"/>
     </row>
@@ -8136,34 +8148,34 @@
     </row>
     <row r="4" spans="1:2" ht="31.5" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" customHeight="1">
@@ -8171,7 +8183,7 @@
         <v>108</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" customHeight="1">
@@ -8179,7 +8191,7 @@
         <v>138</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" customHeight="1">
@@ -8187,7 +8199,7 @@
         <v>29</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="30" customHeight="1">
@@ -8195,7 +8207,7 @@
         <v>105</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1">
@@ -8203,7 +8215,7 @@
         <v>136</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="30" customHeight="1">
@@ -8211,15 +8223,15 @@
         <v>313</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="30" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>